<commit_message>
Updates to game data
</commit_message>
<xml_diff>
--- a/GameHistory.xlsx
+++ b/GameHistory.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e7585a4db9994b00/Documents/src/github/ai/temp-the-middle-helper/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e7585a4db9994b00/Documents/src/github/ai/the-middle-helper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{57280AE6-CADC-4BCE-85CC-7D13E39B1D43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74D6BB18-EB53-4893-A0D2-C69B7391980F}"/>
+  <xr:revisionPtr revIDLastSave="361" documentId="8_{57280AE6-CADC-4BCE-85CC-7D13E39B1D43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD3EB58C-4530-4F98-BB8C-A79F41C66117}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{8A93F8A8-521D-4286-BBCC-988A47D39300}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="181">
   <si>
     <t>Date</t>
   </si>
@@ -65,9 +65,6 @@
     <t>Category</t>
   </si>
   <si>
-    <t>Bovine</t>
-  </si>
-  <si>
     <t>Chalk</t>
   </si>
   <si>
@@ -111,6 +108,480 @@
   </si>
   <si>
     <t>Superb</t>
+  </si>
+  <si>
+    <t>Beside</t>
+  </si>
+  <si>
+    <t>Nephew</t>
+  </si>
+  <si>
+    <t>Overall</t>
+  </si>
+  <si>
+    <t>Sausage</t>
+  </si>
+  <si>
+    <t>Split</t>
+  </si>
+  <si>
+    <t>Free</t>
+  </si>
+  <si>
+    <t>Highlight</t>
+  </si>
+  <si>
+    <t>Dairy</t>
+  </si>
+  <si>
+    <t>Efficient</t>
+  </si>
+  <si>
+    <t>Antenna</t>
+  </si>
+  <si>
+    <t>Birth</t>
+  </si>
+  <si>
+    <t>Across</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>Casual</t>
+  </si>
+  <si>
+    <t>Cough</t>
+  </si>
+  <si>
+    <t>Bliss</t>
+  </si>
+  <si>
+    <t>Chosen</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>Cupboard</t>
+  </si>
+  <si>
+    <t>Entity</t>
+  </si>
+  <si>
+    <t>Gallon</t>
+  </si>
+  <si>
+    <t>Same</t>
+  </si>
+  <si>
+    <t>Specific</t>
+  </si>
+  <si>
+    <t>Recovery</t>
+  </si>
+  <si>
+    <t>Seen</t>
+  </si>
+  <si>
+    <t>Bedroom</t>
+  </si>
+  <si>
+    <t>Cave</t>
+  </si>
+  <si>
+    <t>Substance</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>Equity</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Recruit</t>
+  </si>
+  <si>
+    <t>Sell</t>
+  </si>
+  <si>
+    <t>Reward</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Percent</t>
+  </si>
+  <si>
+    <t>Procedure</t>
+  </si>
+  <si>
+    <t>Suspend</t>
+  </si>
+  <si>
+    <t>Turtle</t>
+  </si>
+  <si>
+    <t>Snake</t>
+  </si>
+  <si>
+    <t>Symphony</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>Circular</t>
+  </si>
+  <si>
+    <t>Express</t>
+  </si>
+  <si>
+    <t>Gown</t>
+  </si>
+  <si>
+    <t>Forecast</t>
+  </si>
+  <si>
+    <t>Helpful</t>
+  </si>
+  <si>
+    <t>Comedian</t>
+  </si>
+  <si>
+    <t>Desk</t>
+  </si>
+  <si>
+    <t>Describe</t>
+  </si>
+  <si>
+    <t>Entrance</t>
+  </si>
+  <si>
+    <t>cheese</t>
+  </si>
+  <si>
+    <t>Chicken</t>
+  </si>
+  <si>
+    <t>chomp</t>
+  </si>
+  <si>
+    <t>calf</t>
+  </si>
+  <si>
+    <t>combat</t>
+  </si>
+  <si>
+    <t>Acute</t>
+  </si>
+  <si>
+    <t>Perfect</t>
+  </si>
+  <si>
+    <t>Process</t>
+  </si>
+  <si>
+    <t>Successor</t>
+  </si>
+  <si>
+    <t>Tray</t>
+  </si>
+  <si>
+    <t>Superstar</t>
+  </si>
+  <si>
+    <t>Trophy</t>
+  </si>
+  <si>
+    <t>Patient</t>
+  </si>
+  <si>
+    <t>Premiere</t>
+  </si>
+  <si>
+    <t>Berry</t>
+  </si>
+  <si>
+    <t>Chamber</t>
+  </si>
+  <si>
+    <t>Architect</t>
+  </si>
+  <si>
+    <t>Boundary</t>
+  </si>
+  <si>
+    <t>Thread</t>
+  </si>
+  <si>
+    <t>Unhealthy</t>
+  </si>
+  <si>
+    <t>Bicycle</t>
+  </si>
+  <si>
+    <t>Chef</t>
+  </si>
+  <si>
+    <t>Literal</t>
+  </si>
+  <si>
+    <t>Motorcycle</t>
+  </si>
+  <si>
+    <t>Forever</t>
+  </si>
+  <si>
+    <t>Heritage</t>
+  </si>
+  <si>
+    <t>Tank</t>
+  </si>
+  <si>
+    <t>Umbrella</t>
+  </si>
+  <si>
+    <t>Itself</t>
+  </si>
+  <si>
+    <t>Mango</t>
+  </si>
+  <si>
+    <t>Mint</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Ship</t>
+  </si>
+  <si>
+    <t>Subway</t>
+  </si>
+  <si>
+    <t>Asleep</t>
+  </si>
+  <si>
+    <t>Broken</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Physician</t>
+  </si>
+  <si>
+    <t>Vase</t>
+  </si>
+  <si>
+    <t>Yourself</t>
+  </si>
+  <si>
+    <t>Math</t>
+  </si>
+  <si>
+    <t>Niece</t>
+  </si>
+  <si>
+    <t>Nobody</t>
+  </si>
+  <si>
+    <t>Overtime</t>
+  </si>
+  <si>
+    <t>Indent</t>
+  </si>
+  <si>
+    <t>Interface</t>
+  </si>
+  <si>
+    <t>Lounge</t>
+  </si>
+  <si>
+    <t>Cross</t>
+  </si>
+  <si>
+    <t>Drawer</t>
+  </si>
+  <si>
+    <t>Bark</t>
+  </si>
+  <si>
+    <t>Careful</t>
+  </si>
+  <si>
+    <t>Practical</t>
+  </si>
+  <si>
+    <t>Regular</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Nonprofit</t>
+  </si>
+  <si>
+    <t>Miracle</t>
+  </si>
+  <si>
+    <t>Noon</t>
+  </si>
+  <si>
+    <t>Remember</t>
+  </si>
+  <si>
+    <t>Shall</t>
+  </si>
+  <si>
+    <t>Usage</t>
+  </si>
+  <si>
+    <t>Zero</t>
+  </si>
+  <si>
+    <t>Basin</t>
+  </si>
+  <si>
+    <t>Cartoon</t>
+  </si>
+  <si>
+    <t>Fluid</t>
+  </si>
+  <si>
+    <t>Hedge</t>
+  </si>
+  <si>
+    <t>Bone</t>
+  </si>
+  <si>
+    <t>Circus</t>
+  </si>
+  <si>
+    <t>Bird</t>
+  </si>
+  <si>
+    <t>Chip</t>
+  </si>
+  <si>
+    <t>Spray</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Argue</t>
+  </si>
+  <si>
+    <t>Brake</t>
+  </si>
+  <si>
+    <t>Amber</t>
+  </si>
+  <si>
+    <t>Become</t>
+  </si>
+  <si>
+    <t>Coat</t>
+  </si>
+  <si>
+    <t>Deliver</t>
+  </si>
+  <si>
+    <t>Unless</t>
+  </si>
+  <si>
+    <t>Would</t>
+  </si>
+  <si>
+    <t>Entry</t>
+  </si>
+  <si>
+    <t>Game</t>
+  </si>
+  <si>
+    <t>Care</t>
+  </si>
+  <si>
+    <t>Cord</t>
+  </si>
+  <si>
+    <t>Fill</t>
+  </si>
+  <si>
+    <t>Hallway</t>
+  </si>
+  <si>
+    <t>Gateway</t>
+  </si>
+  <si>
+    <t>Hunt</t>
+  </si>
+  <si>
+    <t>Engineer</t>
+  </si>
+  <si>
+    <t>Funnel</t>
+  </si>
+  <si>
+    <t>Foam</t>
+  </si>
+  <si>
+    <t>Helicopter</t>
+  </si>
+  <si>
+    <t>Refuge</t>
+  </si>
+  <si>
+    <t>Sensor</t>
+  </si>
+  <si>
+    <t>Referee</t>
+  </si>
+  <si>
+    <t>Send</t>
+  </si>
+  <si>
+    <t>Inspector</t>
+  </si>
+  <si>
+    <t>Kangaroo</t>
+  </si>
+  <si>
+    <t>Melody</t>
+  </si>
+  <si>
+    <t>Favor</t>
+  </si>
+  <si>
+    <t>Guardian</t>
+  </si>
+  <si>
+    <t>Catch</t>
+  </si>
+  <si>
+    <t>Could</t>
+  </si>
+  <si>
+    <t>Logic</t>
+  </si>
+  <si>
+    <t>Announce</t>
+  </si>
+  <si>
+    <t>Bigger</t>
+  </si>
+  <si>
+    <t>Sandy</t>
+  </si>
+  <si>
+    <t>Spend</t>
   </si>
 </sst>
 </file>
@@ -154,12 +625,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -494,14 +964,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09861D7D-33BD-48B2-A348-D79B9CC39536}">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:M89"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -515,123 +985,1005 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="1">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A2" s="3">
         <v>46263</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="H2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I2" t="s">
+        <v>118</v>
+      </c>
+      <c r="K2" t="s">
+        <v>77</v>
+      </c>
+      <c r="L2">
+        <v>-6761</v>
+      </c>
+      <c r="M2">
+        <f>110000+L2</f>
+        <v>103239</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>46260</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="1">
-        <v>46260</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="1">
+      <c r="K3" t="s">
+        <v>74</v>
+      </c>
+      <c r="L3">
+        <v>-508</v>
+      </c>
+      <c r="M3">
+        <f>110000+L3</f>
+        <v>109492</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
         <v>46254</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="K4" t="s">
+        <v>75</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <f>110000+L4</f>
+        <v>110000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>46258</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="K5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L5">
+        <v>975</v>
+      </c>
+      <c r="M5">
+        <f>110000+L5</f>
+        <v>110975</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" s="3">
+        <v>46250</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" s="3">
+        <v>46237</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" s="3">
+        <v>46205</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A9" s="3">
+        <v>46190</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
+        <v>46261</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A11" s="3">
+        <v>46251</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
+        <v>46262</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>46223</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A14" s="3">
+        <v>46188</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A15" s="1">
+        <v>46197</v>
+      </c>
+      <c r="B15" t="s">
+        <v>147</v>
+      </c>
+      <c r="C15" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1">
+        <v>46273</v>
+      </c>
+      <c r="B16" t="s">
+        <v>177</v>
+      </c>
+      <c r="C16" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="1">
+        <v>46214</v>
+      </c>
+      <c r="B19" t="s">
+        <v>90</v>
+      </c>
+      <c r="C19" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="1">
+        <v>46196</v>
+      </c>
+      <c r="B20" t="s">
+        <v>145</v>
+      </c>
+      <c r="C20" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="1">
+        <v>46189</v>
+      </c>
+      <c r="B21" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" s="1">
+        <v>46265</v>
+      </c>
+      <c r="B22" t="s">
+        <v>135</v>
+      </c>
+      <c r="C22" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="1">
+        <v>46243</v>
+      </c>
+      <c r="B23" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="1">
+        <v>46213</v>
+      </c>
+      <c r="B24" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="1">
+        <v>46254</v>
+      </c>
+      <c r="B25" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" s="1">
+        <v>46216</v>
+      </c>
+      <c r="B26" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="1">
+        <v>46194</v>
+      </c>
+      <c r="B27" t="s">
+        <v>141</v>
+      </c>
+      <c r="C27" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" s="1">
+        <v>46248</v>
+      </c>
+      <c r="B28" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" s="1">
+        <v>46204</v>
+      </c>
+      <c r="B29" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="1">
+        <v>46193</v>
+      </c>
+      <c r="B30" t="s">
+        <v>139</v>
+      </c>
+      <c r="C30" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" s="1">
+        <v>46203</v>
+      </c>
+      <c r="B31" t="s">
+        <v>155</v>
+      </c>
+      <c r="C31" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" s="1">
+        <v>46249</v>
+      </c>
+      <c r="B32" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="1">
+        <v>46271</v>
+      </c>
+      <c r="B33" t="s">
+        <v>174</v>
+      </c>
+      <c r="C33" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="1">
+        <v>46247</v>
+      </c>
+      <c r="B34" t="s">
+        <v>40</v>
+      </c>
+      <c r="C34" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" s="1">
+        <v>46198</v>
+      </c>
+      <c r="B35" t="s">
+        <v>149</v>
+      </c>
+      <c r="C35" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="1">
+        <v>46208</v>
+      </c>
+      <c r="B36" t="s">
+        <v>70</v>
+      </c>
+      <c r="C36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" s="1">
+        <v>46234</v>
+      </c>
+      <c r="B37" t="s">
+        <v>161</v>
+      </c>
+      <c r="C37" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="1">
+        <v>46246</v>
+      </c>
+      <c r="B38" t="s">
+        <v>42</v>
+      </c>
+      <c r="C38" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" s="1">
+        <v>46201</v>
+      </c>
+      <c r="B39" t="s">
+        <v>153</v>
+      </c>
+      <c r="C39" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" s="1">
+        <v>46241</v>
+      </c>
+      <c r="B40" t="s">
+        <v>52</v>
+      </c>
+      <c r="C40" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" s="1">
+        <v>46206</v>
+      </c>
+      <c r="B41" t="s">
+        <v>66</v>
+      </c>
+      <c r="C41" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" s="1">
+        <v>46270</v>
+      </c>
+      <c r="B42" t="s">
+        <v>172</v>
+      </c>
+      <c r="C42" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" s="1">
+        <v>46232</v>
+      </c>
+      <c r="B43" t="s">
+        <v>157</v>
+      </c>
+      <c r="C43" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" s="1">
+        <v>46264</v>
+      </c>
+      <c r="B44" t="s">
+        <v>137</v>
+      </c>
+      <c r="C44" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" s="1">
+        <v>46268</v>
+      </c>
+      <c r="B45" t="s">
+        <v>163</v>
+      </c>
+      <c r="C45" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" s="1">
+        <v>46207</v>
+      </c>
+      <c r="B46" t="s">
+        <v>68</v>
+      </c>
+      <c r="C46" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" s="1">
+        <v>46218</v>
+      </c>
+      <c r="B47" t="s">
+        <v>98</v>
+      </c>
+      <c r="C47" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" s="1">
+        <v>46233</v>
+      </c>
+      <c r="B48" t="s">
+        <v>159</v>
+      </c>
+      <c r="C48" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49" s="1">
+        <v>46272</v>
+      </c>
+      <c r="B49" t="s">
+        <v>169</v>
+      </c>
+      <c r="C49" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" s="1">
+        <v>46202</v>
+      </c>
+      <c r="B50" t="s">
+        <v>119</v>
+      </c>
+      <c r="C50" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" s="1">
+        <v>46220</v>
+      </c>
+      <c r="B51" t="s">
+        <v>102</v>
+      </c>
+      <c r="C51" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" s="1">
+        <v>46269</v>
+      </c>
+      <c r="B52" t="s">
+        <v>170</v>
+      </c>
+      <c r="C52" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A53" s="1">
+        <v>46217</v>
+      </c>
+      <c r="B53" t="s">
+        <v>96</v>
+      </c>
+      <c r="C53" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" s="1">
+        <v>46228</v>
+      </c>
+      <c r="B54" t="s">
+        <v>114</v>
+      </c>
+      <c r="C54" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" s="1">
+        <v>46192</v>
+      </c>
+      <c r="B55" t="s">
+        <v>127</v>
+      </c>
+      <c r="C55" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" s="1">
+        <v>46221</v>
+      </c>
+      <c r="B56" t="s">
+        <v>104</v>
+      </c>
+      <c r="C56" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" s="1">
+        <v>46267</v>
+      </c>
+      <c r="B57" t="s">
+        <v>129</v>
+      </c>
+      <c r="C57" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" s="1">
+        <v>46253</v>
+      </c>
+      <c r="B58" t="s">
+        <v>24</v>
+      </c>
+      <c r="C58" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59" s="1">
+        <v>46231</v>
+      </c>
+      <c r="B59" t="s">
+        <v>116</v>
+      </c>
+      <c r="C59" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60" s="1">
+        <v>46224</v>
+      </c>
+      <c r="B60" t="s">
+        <v>110</v>
+      </c>
+      <c r="C60" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" s="1">
+        <v>46212</v>
+      </c>
+      <c r="B61" t="s">
+        <v>86</v>
+      </c>
+      <c r="C61" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B62" t="s">
+        <v>58</v>
+      </c>
+      <c r="C62" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" s="1">
+        <v>46209</v>
+      </c>
+      <c r="B63" t="s">
+        <v>80</v>
+      </c>
+      <c r="C63" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" s="1">
+        <v>46256</v>
+      </c>
+      <c r="B64" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" s="1">
-        <v>46262</v>
-      </c>
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="1">
-        <v>46261</v>
-      </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="C64" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" s="1">
+        <v>46191</v>
+      </c>
+      <c r="B65" t="s">
+        <v>125</v>
+      </c>
+      <c r="C65" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A66" s="1">
+        <v>46259</v>
+      </c>
+      <c r="B66" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="1">
-        <v>46259</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C66" t="s">
         <v>14</v>
       </c>
-      <c r="C9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="1">
-        <v>46256</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" t="s">
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A67" s="1">
+        <v>46244</v>
+      </c>
+      <c r="B67" t="s">
+        <v>46</v>
+      </c>
+      <c r="C67" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A68" s="1">
+        <v>46240</v>
+      </c>
+      <c r="B68" t="s">
+        <v>54</v>
+      </c>
+      <c r="C68" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A69" s="1">
+        <v>46227</v>
+      </c>
+      <c r="B69" t="s">
+        <v>167</v>
+      </c>
+      <c r="C69" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A70" s="1">
+        <v>46226</v>
+      </c>
+      <c r="B70" t="s">
+        <v>165</v>
+      </c>
+      <c r="C70" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A71" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B71" t="s">
+        <v>131</v>
+      </c>
+      <c r="C71" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A72" s="1">
+        <v>46239</v>
+      </c>
+      <c r="B72" t="s">
+        <v>56</v>
+      </c>
+      <c r="C72" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A73" s="1">
+        <v>46245</v>
+      </c>
+      <c r="B73" t="s">
+        <v>44</v>
+      </c>
+      <c r="C73" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A74" s="1">
+        <v>46274</v>
+      </c>
+      <c r="B74" t="s">
+        <v>179</v>
+      </c>
+      <c r="C74" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A75" s="1">
+        <v>46252</v>
+      </c>
+      <c r="B75" t="s">
+        <v>26</v>
+      </c>
+      <c r="C75" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A76" s="1">
+        <v>46222</v>
+      </c>
+      <c r="B76" t="s">
+        <v>106</v>
+      </c>
+      <c r="C76" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A77" s="1">
+        <v>46255</v>
+      </c>
+      <c r="B77" t="s">
+        <v>21</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A78" s="1">
+        <v>46257</v>
+      </c>
+      <c r="B78" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="1">
-        <v>46257</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C78" t="s">
         <v>20</v>
       </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="1">
-        <v>46255</v>
-      </c>
-      <c r="B12" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" t="s">
-        <v>23</v>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A79" s="1">
+        <v>46235</v>
+      </c>
+      <c r="B79" t="s">
+        <v>62</v>
+      </c>
+      <c r="C79" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A80" s="1">
+        <v>46195</v>
+      </c>
+      <c r="B80" t="s">
+        <v>143</v>
+      </c>
+      <c r="C80" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A81" s="1">
+        <v>46242</v>
+      </c>
+      <c r="B81" t="s">
+        <v>50</v>
+      </c>
+      <c r="C81" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A82" s="1">
+        <v>46210</v>
+      </c>
+      <c r="B82" t="s">
+        <v>82</v>
+      </c>
+      <c r="C82" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A83" s="1">
+        <v>46211</v>
+      </c>
+      <c r="B83" t="s">
+        <v>84</v>
+      </c>
+      <c r="C83" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A84" s="1">
+        <v>46236</v>
+      </c>
+      <c r="B84" t="s">
+        <v>60</v>
+      </c>
+      <c r="C84" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A85" s="1">
+        <v>46219</v>
+      </c>
+      <c r="B85" t="s">
+        <v>100</v>
+      </c>
+      <c r="C85" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A86" s="1">
+        <v>46215</v>
+      </c>
+      <c r="B86" t="s">
+        <v>92</v>
+      </c>
+      <c r="C86" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A87" s="1">
+        <v>46200</v>
+      </c>
+      <c r="B87" t="s">
+        <v>151</v>
+      </c>
+      <c r="C87" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A88" s="1">
+        <v>46199</v>
+      </c>
+      <c r="B88" t="s">
+        <v>133</v>
+      </c>
+      <c r="C88" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A89" s="1">
+        <v>46225</v>
+      </c>
+      <c r="B89" t="s">
+        <v>112</v>
+      </c>
+      <c r="C89" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A18:C89">
+    <sortCondition ref="B18:B89"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>